<commit_message>
B&N rev13 WIP: RFI-13 / RFI-22 revised-by-RFI-55 notes (BE-47)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBQT8jCVU6KW8QmKhZS83
</commit_message>
<xml_diff>
--- a/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev13.xlsx
+++ b/cache_proyectos/barnes_noble/takeoff_work/etapas/8_excel/Barnes_Noble_ColoradoSprings_Takeoff_FINAL_rev13.xlsx
@@ -1600,7 +1600,7 @@
     <t xml:space="preserve">CLOSED - estimator decision 2026-10-27: FRP-1 in our scope. N/SHEET: A-510; 1-4/A-226B; 9-12/A-200.</t>
   </si>
   <si>
-    <t xml:space="preserve">Applied: FRP + 1,030.64 SF (Cafe Work Room 875.20 + Janitor 155.44) + PVC trim (J-mold top / bottom + inside corners).</t>
+    <t xml:space="preserve">Applied: FRP + 1,030.64 SF (Cafe Work Room 875.20 + Janitor 155.44) + PVC trim (J-mold top / bottom + inside corners). Revised by RFI-55 (estimator decision 2026-10-28): Work Room FRP 852.20 SF (finished dimensions, 1/A-221); PVC trim per real corners / edges + division bars.</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-14</t>
@@ -1678,7 +1678,7 @@
     <t xml:space="preserve">CLOSED - estimator decision 2026-10-27: One face of types 3 / 4 (122.32 LF) = 5/8" FRT plywood + FRP (A-410 building dept note: all plywood FRT). N/SHEET: 3/A-410; 4/A-410.</t>
   </si>
   <si>
-    <t xml:space="preserve">Applied: 5/8" FRT plywood + 936.74 SF, FRP + 936.74 SF, 5/8" Type X - 936.74 SF on that face, PVC trim + 244.64 LF.</t>
+    <t xml:space="preserve">Applied: 5/8" FRT plywood + 936.74 SF, FRP + 936.74 SF, 5/8" Type X - 936.74 SF on that face, PVC trim + 244.64 LF. Revised by RFI-55 (estimator decision 2026-10-28): types 3 / 4 PVC 154.32 LF (hourglass cap corners take the metal corner guard) + division bars 167 LF.</t>
   </si>
   <si>
     <t xml:space="preserve">RFI-23</t>

</xml_diff>